<commit_message>
feat(schema): add BlockGeometry and TVSGeometry worksheets with backward compatibility
Add BlockGeometry and TVSGeometry worksheets to the schema registry and templates,
mark legacy geometry columns as deprecated, implement dual-geometry precedence with
warnings, and enforce sequence, link, and physical continuity validations.
</commit_message>
<xml_diff>
--- a/templates/HEADWAY_ANALYSIS_v1.0.xlsx
+++ b/templates/HEADWAY_ANALYSIS_v1.0.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="85" customWidth="1" min="1" max="1"/>
@@ -585,17 +585,24 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr"/>
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>7. For multi-link signalling blocks or TVS sections, define spatial geometry intervals in the 'BlockGeometry' or 'TVSGeometry' worksheet with sequential numbering.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>WORKSHEET INVENTORY:</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>• AnalysisSettings: Simulation analysis run specifications</t>
         </is>

</xml_diff>

<commit_message>
feat(data): add performance_factor to canonical models, excel registry, and validation
- Add performance_factor and performance_factor_source to AnalysisConfig
- Add default_performance_factor to Scenario and ScenarioDefinition
- Add ColumnDef range constraints [0.5, 1.0] and schema columns
- Enforce ERR_FIELD_RANGE in importer and validator
- Implement precedence hierarchy in converter: analysis row > scenario default > 1.0
- Regenerate standard Excel templates and update JSON schemas
</commit_message>
<xml_diff>
--- a/templates/HEADWAY_ANALYSIS_v1.0.xlsx
+++ b/templates/HEADWAY_ANALYSIS_v1.0.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="85" customWidth="1" min="1" max="1"/>
@@ -592,17 +592,24 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr"/>
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>8. PERFORMANCE_FACTOR: Fraction of nominal traction and service braking available to the train. 1.0 = 100% (full performance), 0.95 = 95%. Does not affect protection braking. Default 1.0 if blank.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>WORKSHEET INVENTORY:</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>• AnalysisSettings: Simulation analysis run specifications</t>
         </is>
@@ -733,7 +740,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -744,8 +751,9 @@
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="23" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -791,10 +799,15 @@
       </c>
       <c r="I1" s="8" t="inlineStr">
         <is>
+          <t>PERFORMANCE_FACTOR</t>
+        </is>
+      </c>
+      <c r="J1" s="8" t="inlineStr">
+        <is>
           <t>REF_LINK_ID</t>
         </is>
       </c>
-      <c r="J1" s="8" t="inlineStr">
+      <c r="K1" s="8" t="inlineStr">
         <is>
           <t>REF_OFFSET_M</t>
         </is>
@@ -848,6 +861,11 @@
       </c>
       <c r="J2" s="9" t="inlineStr">
         <is>
+          <t>(Optional)</t>
+        </is>
+      </c>
+      <c r="K2" s="9" t="inlineStr">
+        <is>
           <t>[m]</t>
         </is>
       </c>
@@ -885,12 +903,15 @@
       <c r="H3" s="10" t="n">
         <v>30</v>
       </c>
-      <c r="I3" s="10" t="inlineStr">
+      <c r="I3" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" s="10" t="inlineStr">
         <is>
           <t>LNK_01</t>
         </is>
       </c>
-      <c r="J3" s="10" t="n">
+      <c r="K3" s="10" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>